<commit_message>
Adding new punishments in documents to test if bot works
</commit_message>
<xml_diff>
--- a/projekt/data/taryfikator.xlsx
+++ b/projekt/data/taryfikator.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marcin\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marcin\Documents\Zadania - studia\PythonLabs\AAP_LAB_TASKS\projekt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79C2F290-D3F8-40AF-AEAC-82CE8E77DED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D978FE3-9509-44EC-89BB-EF213F24373F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F84B3F9F-CC52-44E9-8FEE-3FECB286A998}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>przewinienie</t>
   </si>
@@ -62,7 +62,19 @@
     <t>reklama</t>
   </si>
   <si>
-    <t>ban 7 dni</t>
+    <t>ban</t>
+  </si>
+  <si>
+    <t>popieranie SCT w Krakowie</t>
+  </si>
+  <si>
+    <t>kick</t>
+  </si>
+  <si>
+    <t>mute 2137h</t>
+  </si>
+  <si>
+    <t>scam links</t>
   </si>
 </sst>
 </file>
@@ -450,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D804EAD0-F4FB-46F7-8991-F4D2D6C5BCDC}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -485,6 +497,22 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Upgrading rag to better check words from documents
</commit_message>
<xml_diff>
--- a/projekt/data/taryfikator.xlsx
+++ b/projekt/data/taryfikator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marcin\Documents\Zadania - studia\PythonLabs\AAP_LAB_TASKS\projekt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D978FE3-9509-44EC-89BB-EF213F24373F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B743E582-022A-489A-ABC9-5DF1919E37B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F84B3F9F-CC52-44E9-8FEE-3FECB286A998}"/>
   </bookViews>
@@ -74,7 +74,7 @@
     <t>mute 2137h</t>
   </si>
   <si>
-    <t>scam links</t>
+    <t>wysyłanie scamowych linków</t>
   </si>
 </sst>
 </file>
@@ -505,7 +505,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Fixing taryfikator document to be good compared to regulamin
</commit_message>
<xml_diff>
--- a/projekt/data/taryfikator.xlsx
+++ b/projekt/data/taryfikator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marcin\Documents\Zadania - studia\PythonLabs\AAP_LAB_TASKS\projekt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B743E582-022A-489A-ABC9-5DF1919E37B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A298C343-BF65-4E46-BF3B-671FB42DFF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F84B3F9F-CC52-44E9-8FEE-3FECB286A998}"/>
   </bookViews>
@@ -47,34 +47,34 @@
     <t>kara</t>
   </si>
   <si>
-    <t>spam</t>
-  </si>
-  <si>
     <t>mute 2h</t>
   </si>
   <si>
-    <t>obraza użytkownika</t>
-  </si>
-  <si>
     <t>mute 24h</t>
   </si>
   <si>
-    <t>reklama</t>
-  </si>
-  <si>
     <t>ban</t>
   </si>
   <si>
-    <t>popieranie SCT w Krakowie</t>
-  </si>
-  <si>
     <t>kick</t>
   </si>
   <si>
     <t>mute 2137h</t>
   </si>
   <si>
-    <t>wysyłanie scamowych linków</t>
+    <t>Reklama innych serwerów Discord</t>
+  </si>
+  <si>
+    <t>Wysyłanie scamowych linków</t>
+  </si>
+  <si>
+    <t>Promowanie SCT w Krakowie</t>
+  </si>
+  <si>
+    <t>Obrażanie innych użytkowników</t>
+  </si>
+  <si>
+    <t>Spam</t>
   </si>
 </sst>
 </file>
@@ -120,13 +120,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -474,43 +477,43 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="5" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>11</v>
+      <c r="A6" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>